<commit_message>
Update testimonials data file and deploy
</commit_message>
<xml_diff>
--- a/public/testimonials.xlsx
+++ b/public/testimonials.xlsx
@@ -1,42 +1,169 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="M:\For Other\fehed\Tech\TechInnoSphere-Single\TechInnoSphere\public\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBFA349B-1094-4BA9-BCFE-F2B3F5B0E837}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="40">
+  <si>
+    <t>Client Name</t>
+  </si>
+  <si>
+    <t>Designation</t>
+  </si>
+  <si>
+    <t>Company</t>
+  </si>
+  <si>
+    <t>Location</t>
+  </si>
+  <si>
+    <t>Feedback</t>
+  </si>
+  <si>
+    <t>Rating</t>
+  </si>
+  <si>
+    <t>Client Photo</t>
+  </si>
+  <si>
+    <t>Related Project</t>
+  </si>
+  <si>
+    <t>Operations Head</t>
+  </si>
+  <si>
+    <t>Shahji Shipping LLC</t>
+  </si>
+  <si>
+    <t>Director</t>
+  </si>
+  <si>
+    <t>Ace Consultants</t>
+  </si>
+  <si>
+    <t>Dubai, UAE</t>
+  </si>
+  <si>
+    <t>TechInnoSphere transformed our logistics operations.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/uc?export=view&amp;id=1qAjHhZgyhfFGQb2L7I5sGi1LPYwRDnlv</t>
+  </si>
+  <si>
+    <t>Toronto, Canada</t>
+  </si>
+  <si>
+    <t>Fast, modern, and highly secure.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/uc?export=view&amp;id=1j3JYusoN2Mrps6y1gNO8VvNMXdOeRQKf</t>
+  </si>
+  <si>
+    <t>Kira Ledgers</t>
+  </si>
+  <si>
+    <t>Vienna, Austria</t>
+  </si>
+  <si>
+    <t>The AI-generated visuals were highly realistic and helped us create professional fashion content quickly and cost-effectively.</t>
+  </si>
+  <si>
+    <t>Founder</t>
+  </si>
+  <si>
+    <t>Sweezen Foundation</t>
+  </si>
+  <si>
+    <t>Mumbai, India</t>
+  </si>
+  <si>
+    <t>The platform streamlined our donation and volunteer management processes, making it easier to engage supporters worldwide and significantly grow our fundraising efforts.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/uc?export=view&amp;id=1cfjXF15f_f6uypHBRy6y5OkzS8PsqwPa</t>
+  </si>
+  <si>
+    <t>Chanakya The Global School</t>
+  </si>
+  <si>
+    <t>Palghar, India</t>
+  </si>
+  <si>
+    <t>The LMS and ERP solution transformed our academic operations, ensuring seamless online learning and uninterrupted examinations for thousands of students.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/uc?export=view&amp;id=1woZK9XkiUlvvBQHL2s4VUtJEBKZcbXnw</t>
+  </si>
+  <si>
+    <t>PMK Iron &amp; Steel</t>
+  </si>
+  <si>
+    <t>Punjab, India</t>
+  </si>
+  <si>
+    <t>The custom ERP and IoT integration automated critical workflows, improved inventory accuracy, and completely eliminated manual data entry errors.</t>
+  </si>
+  <si>
+    <t>News AI Videos</t>
+  </si>
+  <si>
+    <t>Delhi, India</t>
+  </si>
+  <si>
+    <t>The AI-powered video generation platform enabled us to produce high-quality news videos within minutes, helping us deliver breaking news faster than ever.</t>
+  </si>
+  <si>
+    <t>Founder &amp; Managing Director</t>
+  </si>
+  <si>
+    <t>Turant RX</t>
+  </si>
+  <si>
+    <t>The platform transformed our pharmacy operations, making medicine ordering and inventory management faster, more accurate, and highly efficient.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/uc?export=view&amp;id=1TUqeKucxkr4dbj4K2F1lsGwlONvlWG--</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -61,17 +188,36 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,90 +542,254 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:H9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11.19921875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.69921875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.09765625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Client Name</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Designation</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Company</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Location</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Feedback</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Rating</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Client Photo</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Related Project</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Rahul Sharma</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Operations Head</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Shahji Shipping LLC</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Dubai</v>
-      </c>
-      <c r="E2" t="str">
-        <v>TechInnoSphere transformed our logistics operations with their enterprise software.</v>
-      </c>
-      <c r="F2">
+    <row r="1" spans="1:8" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G2" t="str">
-        <v/>
-      </c>
-      <c r="H2" t="str">
-        <v>Shahji Shipping LLC</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Sarah Jenkins</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Director</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Ace Consultants</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Canada</v>
-      </c>
-      <c r="E3" t="str">
-        <v>The web platform they built for us is fast, modern, and has significantly improved our client acquisition.</v>
-      </c>
-      <c r="F3">
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="156" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="2">
         <v>5</v>
       </c>
-      <c r="G3" t="str">
-        <v/>
-      </c>
-      <c r="H3" t="str">
-        <v>Ace Consultants</v>
+      <c r="G2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="156" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="2">
+        <v>5</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="265.2" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" s="2">
+        <v>4</v>
+      </c>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="390" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F5" s="2">
+        <v>5</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="312" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" s="2">
+        <v>4</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="374.4" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F7" s="2">
+        <v>5</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="358.8" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F8" s="2">
+        <v>5</v>
+      </c>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="343.2" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F9" s="2">
+        <v>5</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H3"/>
-  </ignoredErrors>
+  <hyperlinks>
+    <hyperlink ref="G2" r:id="rId1" xr:uid="{3E4AD545-8503-431F-914B-048C1937BEF0}"/>
+    <hyperlink ref="G3" r:id="rId2" xr:uid="{4697C8C2-A03B-4709-890F-B43F151D6458}"/>
+    <hyperlink ref="G5" r:id="rId3" xr:uid="{BBA29DCB-B718-40B2-83CE-E1AB0F01137D}"/>
+    <hyperlink ref="G6" r:id="rId4" xr:uid="{CC5649C5-4E50-45CC-A3B2-D09AAE1485E8}"/>
+    <hyperlink ref="G7" r:id="rId5" xr:uid="{1897BA95-FFE5-409B-BD6C-8B58418D2406}"/>
+    <hyperlink ref="G9" r:id="rId6" xr:uid="{58863B7D-4FCF-4D14-9AAC-65763E8BDF36}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>